<commit_message>
MDM Files modified for CD ROM, RMI TOOL & MNAO DATA EXPORT TOOL
</commit_message>
<xml_diff>
--- a/KaptureConfigs/Environment_Config/Kapture_Environment_Config.xlsx
+++ b/KaptureConfigs/Environment_Config/Kapture_Environment_Config.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,10 +18,10 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Jobs'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Batch Jobs'!$A$1:$M$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Where Configured'!$A$1:$E$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Where Configured'!$A$1:$E$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DB User Switch'!$A$1:$F$9</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -52,8 +53,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="6">
@@ -65,22 +65,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
+        <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,18 +94,17 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFBFBFBF"/>
+        <color rgb="00BFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="FFBFBFBF"/>
+        <color rgb="00BFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="FFBFBFBF"/>
+        <color rgb="00BFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFBFBFBF"/>
+        <color rgb="00BFBFBF"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -147,7 +146,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -511,27 +510,27 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Kapture Environment Config</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-19 by tmp/Environment_Config/build_environment_config.py - edit the script, then regenerate, so the workbook stays the single place for every environment's settings.</t>
+          <t>Generated 2026-10-30 by tmp/Environment_Config/build_environment_config.py - edit the script, then regenerate, so the workbook stays the single place for every environment's settings.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
+      <c r="A3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -554,7 +553,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="25" customHeight="1">
+    <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Batch Jobs - the 8 Kapture batch jobs that replace the InfoManager custom batch jobs: jar, legacy job, what it reads and writes, schedule, port, report folder, delivery, open items.</t>
@@ -583,7 +582,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
+      <c r="A11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -607,7 +606,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
+      <c r="A15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -628,11 +627,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F67"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="5"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -680,7 +681,7 @@
       <c r="E2" s="7" t="n"/>
       <c r="F2" s="7" t="n"/>
     </row>
-    <row r="3" ht="25" customHeight="1">
+    <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>MySQL database</t>
@@ -712,7 +713,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="37.5" customHeight="1">
+    <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>MySQL database</t>
@@ -770,9 +771,9 @@
           <t>kapture_dc</t>
         </is>
       </c>
-      <c r="F5" s="8" t="n"/>
-    </row>
-    <row r="6" ht="25" customHeight="1">
+      <c r="F5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>MySQL database</t>
@@ -804,7 +805,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="25" customHeight="1">
+    <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>MySQL database</t>
@@ -862,7 +863,7 @@
           <t>kapture_dc_dl$#2026</t>
         </is>
       </c>
-      <c r="F8" s="8" t="n"/>
+      <c r="F8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -875,13 +876,13 @@
           <t>Previous MC Dev DB user (retired)</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n"/>
+      <c r="C9" s="8" t="inlineStr"/>
       <c r="D9" s="8" t="inlineStr">
         <is>
           <t>v118433 / mcdev123</t>
         </is>
       </c>
-      <c r="E9" s="8" t="n"/>
+      <c r="E9" s="8" t="inlineStr"/>
       <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Replace everywhere - see sheet 'DB User Switch'.</t>
@@ -920,7 +921,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="62.5" customHeight="1">
+    <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>MySQL database</t>
@@ -1054,7 +1055,7 @@
           <t>8891</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n"/>
+      <c r="F15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1082,7 +1083,7 @@
           <t>http://oclut0142:8891</t>
         </is>
       </c>
-      <c r="F16" s="8" t="n"/>
+      <c r="F16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1142,7 +1143,7 @@
           <t>/kauthor-api/cms-check</t>
         </is>
       </c>
-      <c r="F18" s="8" t="n"/>
+      <c r="F18" s="8" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1234,7 +1235,7 @@
           <t>kauthor</t>
         </is>
       </c>
-      <c r="F21" s="8" t="n"/>
+      <c r="F21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -1262,7 +1263,7 @@
           <t>oclut0142</t>
         </is>
       </c>
-      <c r="F22" s="8" t="n"/>
+      <c r="F22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1276,7 +1277,7 @@
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="7" t="n"/>
     </row>
-    <row r="24" ht="37.5" customHeight="1">
+    <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Content store</t>
@@ -1308,7 +1309,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="50" customHeight="1">
+    <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Content store</t>
@@ -1340,7 +1341,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="62.5" customHeight="1">
+    <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Content store</t>
@@ -1372,7 +1373,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="25" customHeight="1">
+    <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Content store</t>
@@ -1398,7 +1399,7 @@
           <t>/s3kapture/ROOT/resources/sites/KAPTURE/content/library/MAZDA/</t>
         </is>
       </c>
-      <c r="F27" s="8" t="n"/>
+      <c r="F27" s="8" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -1432,7 +1433,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1">
+    <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Source Oracle (migration jobs)</t>
@@ -1444,7 +1445,7 @@
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="7" t="n"/>
     </row>
-    <row r="30" ht="25" customHeight="1">
+    <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Source Oracle (migration jobs)</t>
@@ -1476,7 +1477,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="25" customHeight="1">
+    <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Source Oracle (migration jobs)</t>
@@ -1508,7 +1509,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="25" customHeight="1">
+    <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Source Oracle (migration jobs)</t>
@@ -1540,7 +1541,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="25" customHeight="1">
+    <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Source Oracle (migration jobs)</t>
@@ -1572,7 +1573,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="25" customHeight="1">
+    <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>Source Oracle (migration jobs)</t>
@@ -1616,7 +1617,7 @@
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="7" t="n"/>
     </row>
-    <row r="36" ht="25" customHeight="1">
+    <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>Mail</t>
@@ -1674,9 +1675,9 @@
           <t>TSSOKIMRCA@mazda.ca</t>
         </is>
       </c>
-      <c r="F37" s="8" t="n"/>
-    </row>
-    <row r="38" ht="25" customHeight="1">
+      <c r="F37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>Mail</t>
@@ -1702,9 +1703,9 @@
           <t>vishald@softclouds.com,gauravb@softclouds.com</t>
         </is>
       </c>
-      <c r="F38" s="8" t="n"/>
-    </row>
-    <row r="39" ht="52" customHeight="1">
+      <c r="F38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -1716,7 +1717,7 @@
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="7" t="n"/>
     </row>
-    <row r="40" ht="50" customHeight="1">
+    <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -1748,7 +1749,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="50" customHeight="1">
+    <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -1780,7 +1781,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="62.5" customHeight="1">
+    <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -1812,7 +1813,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="50" customHeight="1">
+    <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -1844,7 +1845,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="50" customHeight="1">
+    <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -1876,7 +1877,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="50" customHeight="1">
+    <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -1908,7 +1909,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="50" customHeight="1">
+    <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -1940,7 +1941,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="50" customHeight="1">
+    <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -1972,7 +1973,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="50" customHeight="1">
+    <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -2004,7 +2005,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="50" customHeight="1">
+    <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -2036,7 +2037,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="50" customHeight="1">
+    <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Kapture batch jobs (replace the InfoManager custom batch jobs)</t>
@@ -2068,7 +2069,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="52" customHeight="1">
+    <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2080,7 +2081,7 @@
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="7" t="n"/>
     </row>
-    <row r="52" ht="50" customHeight="1">
+    <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2101,7 +2102,7 @@
           <t>JDK 25 at /app/java (java.home); 3 standalone core-Java jars (no Spring): extract (cron hourly + RERUN), Run On Demand poller (cron), transfer (started by the extract)</t>
         </is>
       </c>
-      <c r="E52" s="10" t="inlineStr">
+      <c r="E52" s="8" t="inlineStr">
         <is>
           <t>JDK 25 at /app/java (java.home)</t>
         </is>
@@ -2112,7 +2113,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="50" customHeight="1">
+    <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2144,7 +2145,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="50" customHeight="1">
+    <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2176,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="62.5" customHeight="1">
+    <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2208,7 +2209,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="50" customHeight="1">
+    <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2240,7 +2241,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="50" customHeight="1">
+    <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2272,7 +2273,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="87.5" customHeight="1">
+    <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2304,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="50" customHeight="1">
+    <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2336,7 +2337,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="50" customHeight="1">
+    <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2368,7 +2369,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="65" customHeight="1">
+    <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2389,7 +2390,7 @@
           <t>y611172</t>
         </is>
       </c>
-      <c r="E61" s="10" t="inlineStr">
+      <c r="E61" s="8" t="inlineStr">
         <is>
           <t>QA: confirm run user (must have ~/.oci/config)</t>
         </is>
@@ -2400,7 +2401,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="50" customHeight="1">
+    <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2421,7 +2422,7 @@
           <t>0 * * * *    /s3kapture/ROOT/resources/sites/KAPTURE/content/library/MAZDA/MGSS_DATA_EXTRACT/jobs/NewMazdaDataExportTool/run.sh</t>
         </is>
       </c>
-      <c r="E62" s="10" t="inlineStr">
+      <c r="E62" s="8" t="inlineStr">
         <is>
           <t>QA: copied from DEV - confirm</t>
         </is>
@@ -2432,7 +2433,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="75" customHeight="1">
+    <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2453,7 +2454,7 @@
           <t>*/5 * * * *  /s3kapture/ROOT/resources/sites/KAPTURE/content/library/MAZDA/MGSS_DATA_EXTRACT/jobs/NewMazdaDataExportTool/run.sh RERUN</t>
         </is>
       </c>
-      <c r="E63" s="10" t="inlineStr">
+      <c r="E63" s="8" t="inlineStr">
         <is>
           <t>QA: copied from DEV - confirm</t>
         </is>
@@ -2464,7 +2465,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="50" customHeight="1">
+    <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2485,7 +2486,7 @@
           <t>*/5 * * * *  /s3kapture/ROOT/resources/sites/KAPTURE/content/library/MAZDA/MGSS_DATA_EXTRACT/jobs/NewMazdaDataRunOnDemandTool/run.sh</t>
         </is>
       </c>
-      <c r="E64" s="10" t="inlineStr">
+      <c r="E64" s="8" t="inlineStr">
         <is>
           <t>QA: copied from DEV - confirm</t>
         </is>
@@ -2496,7 +2497,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="50" customHeight="1">
+    <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract &amp; Transfer jobs (core Java, cron)</t>
@@ -2517,7 +2518,7 @@
           <t>none - started by the extract as a child process: java -jar transferjob.jar &lt;jobId&gt; &lt;attemptId&gt; &lt;threadId&gt;</t>
         </is>
       </c>
-      <c r="E65" s="10" t="inlineStr">
+      <c r="E65" s="8" t="inlineStr">
         <is>
           <t>none (same as MC Dev)</t>
         </is>
@@ -2540,7 +2541,7 @@
       <c r="E66" s="7" t="n"/>
       <c r="F66" s="7" t="n"/>
     </row>
-    <row r="67" ht="25" customHeight="1">
+    <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
           <t>Application</t>
@@ -2584,7 +2585,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
@@ -2626,7 +2627,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1">
+    <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Job 1</t>
@@ -2658,7 +2659,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="25" customHeight="1">
+    <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Job 2</t>
@@ -2754,7 +2755,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="25" customHeight="1">
+    <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Job 5</t>
@@ -2818,7 +2819,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="25" customHeight="1">
+    <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Job 7</t>
@@ -2850,7 +2851,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="25" customHeight="1">
+    <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Job 8</t>
@@ -2914,7 +2915,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="25" customHeight="1">
+    <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Job 10</t>
@@ -2946,7 +2947,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="25" customHeight="1">
+    <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Job 11</t>
@@ -2991,7 +2992,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -3008,7 +3009,7 @@
     <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
           <t>#</t>
@@ -3075,7 +3076,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="75" customHeight="1">
+    <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
           <t>1</t>
@@ -3142,7 +3143,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="37.5" customHeight="1">
+    <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>2</t>
@@ -3209,7 +3210,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="37.5" customHeight="1">
+    <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>3</t>
@@ -3276,7 +3277,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="37.5" customHeight="1">
+    <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>4</t>
@@ -3343,7 +3344,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="37.5" customHeight="1">
+    <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>5</t>
@@ -3410,7 +3411,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="37.5" customHeight="1">
+    <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>6</t>
@@ -3477,7 +3478,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="37.5" customHeight="1">
+    <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>7</t>
@@ -3544,7 +3545,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="50" customHeight="1">
+    <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>8</t>
@@ -3623,8 +3624,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
@@ -3660,7 +3661,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1">
+    <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
           <t>DMT (dmtgt.war)</t>
@@ -3708,9 +3709,9 @@
           <t>Resource jdbc/cms_datasource: url, username, password</t>
         </is>
       </c>
-      <c r="E3" s="8" t="n"/>
-    </row>
-    <row r="4" ht="25" customHeight="1">
+      <c r="E3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>DMT (dmtgt.war)</t>
@@ -3731,9 +3732,9 @@
           <t>kapture.api.base, kapture.api.email, kapture.api.password, kapture.api.publicIp</t>
         </is>
       </c>
-      <c r="E4" s="8" t="n"/>
-    </row>
-    <row r="5" ht="25" customHeight="1">
+      <c r="E4" s="8" t="inlineStr"/>
+    </row>
+    <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>DMT (dmtgt.war)</t>
@@ -3760,7 +3761,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="87.5" customHeight="1">
+    <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>DMT (dmtgt.war)</t>
@@ -3787,7 +3788,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="25" customHeight="1">
+    <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>MDM (mdmgt.war)</t>
@@ -3814,7 +3815,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="37.5" customHeight="1">
+    <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>MDM (mdmgt.war)</t>
@@ -3841,455 +3842,509 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="25" customHeight="1">
+    <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
+          <t>MDM (mdmgt.war)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>SourceCode_Migrated/MDMKapture/env/&lt;DEV|QA|PROD&gt;/application.properties</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>CD Creation / RMI Export / MNAO Data Export - parallel limits</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>cdrom.max.parallel.jobs = 5, cdrom.copy.parallel.threads = 5, rmitool.max.parallel.jobs = 5, dataexttool.max.parallel.jobs = 5</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Added 2026-10-30, REQUIRED (no default in code). max.parallel.jobs = CD jobs Pending / Processing at once (Schedule refused beyond it; selection-criteria jobs not counted). copy.parallel.threads = files one CD job copies at the same time on /s3kapture (WD / e-WD folders, images). Worst case on the mount = jobs x threads = 25. rmitool / dataexttool .max.parallel.jobs = RMI Export / MNAO Data Export jobs Pending / Processing at once, each tool on its own. Same values in every environment (user 2026-10-30).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>MDM (mdmgt.war) - CD Creation / RMI Export / MNAO Data Export - Kapture link forms</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>SourceCode_Migrated/MDMKapture/env/&lt;DEV|QA|PROD&gt;/application.properties</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Kapture link forms in document content</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>cdrom.innerlink.kapture.pattern, rmitool.innerlink.kapture.pattern, dataexttool.innerlink.kapture.pattern = (?:^|/)content/([A-Za-z]+[0-9]+)(?:[/?#&amp;]|$); cdrom.othermanualink.kapture.mc / .mme.url.pattern = result_mc?question_box= / result_mme?question_box=; rimtool.othermanualink.kapture.mnao / .mc / .mme.url.pattern = result? / result_mc? / result_mme?question_box=; cdrom.wd.reflinks.kapture.pattern = mazdagms3/content/</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Added 2026-10-30, REQUIRED (no default in code). Content loaded by Job 10 / DMT carries Kapture links (content/&lt;id&gt;, result_mc?question_box=...); the tools handle them BESIDES the InfoManager forms (rmitool / dataexttool.innerlink.url, rimtool.othermanualink.*), as the Bulk Extract job does. Document link -&gt; exported document (CD: &lt;id&gt;.html), other manual link -&gt; its text, WD window.js / voltage maps (CD) -&gt; ../sm_doc/&lt;id&gt;.html. Same values in every environment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
           <t>AssetsTool (assetstool.war)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>SourceCode_Migrated/AssetsToolKapture/env/&lt;DEV|QA|PROD&gt;/application.properties</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Content store</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>OK_ASSETS_PATH, wsl.default.user, ERROR_REDIRECT_PATH</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>No database, no context.xml.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>DMT, MDM, AssetsTool - logs</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>SourceCode_Migrated/&lt;app&gt;/env/&lt;DEV|QA|PROD&gt;/log.properties</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Log folder</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>log_root_location</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>${catalina.base}/logs/DMT | MDM | AssetsTool (Tomcat's local logs folder) on DEV / QA / PROD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="75" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>DMT, MDM, AssetsTool - build</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>SourceCode_Migrated/&lt;app&gt;/build.bat</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Per-environment WAR</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>build.bat LOCAL | DEV | QA | PROD -&gt; &lt;app&gt;/dist/&lt;ENV&gt;/&lt;war&gt;</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>build.bat LOCAL | DEV | QA | PROD packages env/&lt;ENV&gt;/ (LOCAL = src/ + WebContent/META-INF/context.xml). PROD: fill every __TBC__ first - the build refuses while one is left. env/EnvConfigCheck.java stops the build when a src/application.properties key is missing from env/&lt;ENV&gt;/. META-INF/build-env.txt inside the WAR names the environment. Added 2026-10-14.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
+          <t>DMT, MDM, AssetsTool - logs</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>SourceCode_Migrated/&lt;app&gt;/env/&lt;DEV|QA|PROD&gt;/log.properties</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Log folder</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>log_root_location</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>${catalina.base}/logs/DMT | MDM | AssetsTool (Tomcat's local logs folder) on DEV / QA / PROD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>DMT, MDM, AssetsTool - build</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>SourceCode_Migrated/&lt;app&gt;/build.bat</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Per-environment WAR</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>build.bat LOCAL | DEV | QA | PROD -&gt; &lt;app&gt;/dist/&lt;ENV&gt;/&lt;war&gt;</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>build.bat LOCAL | DEV | QA | PROD packages env/&lt;ENV&gt;/ (LOCAL = src/ + WebContent/META-INF/context.xml). PROD: fill every __TBC__ first - the build refuses while one is left. env/EnvConfigCheck.java stops the build when a src/application.properties key is missing from env/&lt;ENV&gt;/. META-INF/build-env.txt inside the WAR names the environment. Added 2026-10-14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
           <t>Job 11 ContentActivityImportJob</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>SourceCode_Migrated/ContentActivityImportJob/application_vdi.properties</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>DB - kapture_dc</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>activity.db.url, activity.db.user, activity.db.password</t>
         </is>
       </c>
-      <c r="E12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Job 11 ContentActivityImportJob</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>SourceCode_Migrated/ContentActivityImportJob/application_vdi.properties</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>DB - kapture_cms_db</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>activity.cms.db.url, activity.cms.db.user, activity.cms.db.password</t>
         </is>
       </c>
-      <c r="E13" s="8" t="n"/>
-    </row>
-    <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Job 11 ContentActivityImportJob</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>SourceCode_Migrated/ContentActivityImportJob/application_vdi.properties</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Kapture API</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>kapture.api.base, kapture.api.email, kapture.api.password, kapture.api.publicIp</t>
         </is>
       </c>
-      <c r="E14" s="8" t="n"/>
-    </row>
-    <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Jobs 9 / 10 ContentImportJob, ContentBulkImportJob</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>SourceCode_Migrated/&lt;job&gt;/application.properties</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>DB + Kapture API</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>content.import.db.url / .user / .password, kapture.api.*</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>content.import.db.url / .user / .password, kapture.api.*, Job 10 content.import.path.replace.WIRING_DIAGRAMS.from / .to (same in every environment)</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Repo copies carry SC Dev values; the VDI copies carry MC Dev.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Jobs 1-8, ContentPathScanner / Updater</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>SourceCode_Migrated/&lt;job&gt;/application.properties</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>DB (MySQL + Oracle)</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>jdbc.mysql.kapture_dc.*, jdbc.oracle.*</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Repo copies carry workstation values; set the server values on the VDI copy.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="37.5" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>IM batch job rumvinmapping (rumvinmapping.jar)</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>SourceKapture_Batches/rum-vin-mapping/dist/conf/application.properties -&gt; &lt;job folder&gt;/conf/application.properties</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>DB - kapture_dc</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>spring.datasource.url, spring.datasource.username, spring.datasource.password (or env SPRING_DATASOURCE_PASSWORD)</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Added 2026-10-13. Standalone Spring Boot jar, own connection pool (no JNDI). Shipped file = MC Dev values, password blank.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="37.5" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>IM batch job rumvinmapping (rumvinmapping.jar)</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>&lt;job folder&gt;/conf/application.properties</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Run history tables</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>spring.batch.jdbc.table-prefix=KM_CUSTOM_BATCH_, batch.schema.auto-create</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>KM_CUSTOM_BATCH_* in kapture_dc, shared by all IM batch jobs; created by the first job start (needs CREATE once) or by db/km_custom_batch_metadata_mysql.sql.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="50" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>IM batch job rumvinmapping (rumvinmapping.jar)</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>&lt;job folder&gt;/conf/application.properties</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Folders, mail, run mode, logs</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>rumvin.source.dir / archive.dir / reports.dir / reports.web.path, notification.smtp.*, batch.run.mode (once / service), batch.job.cron, logging.file.name + logging.logback.rollingpolicy.*</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Linux source / archive folders still to be confirmed. Mail: smtp.mazdausa.com port 25, no auth (as MDM).</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="100" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>IM batch jobs mmevcesilabelsupdate, carlinenotification, siinnerlinksidentification, viewcontentmcsidatamanagement, viewcontentvinsidatamanagement, viewcontentsidatamanagement, viewcontentmmedatamanagement</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>SourceKapture_Batches/&lt;module&gt;/dist/conf/application.properties -&gt; &lt;job folder&gt;/conf/application.properties</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>DB - kapture_dc</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>spring.datasource.url, spring.datasource.username, spring.datasource.password (or env SPRING_DATASOURCE_PASSWORD)</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>Added 2026-10-13. Same layout as rumvinmapping: standalone Spring Boot jar, own connection pool (no JNDI). Shipped files carry MC Dev values, passwords blank.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="100" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>IM batch jobs mmevcesilabelsupdate, carlinenotification, siinnerlinksidentification, viewcontentmcsidatamanagement, viewcontentvinsidatamanagement, viewcontentsidatamanagement, viewcontentmmedatamanagement</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>SourceKapture_Batches/&lt;module&gt;/dist/conf/application.properties -&gt; &lt;job folder&gt;/conf/application.properties</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>DB - kapture_cms_db (read only)</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>cms.datasource.url, cms.datasource.username, cms.datasource.password (or env CMS_DATASOURCE_PASSWORD)</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>All of them except mmevcesilabelsupdate. Same server and account as kapture_dc (kapture_dc_dl, SELECT on kapture_cms_db).</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="100" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>IM batch jobs mmevcesilabelsupdate, carlinenotification, siinnerlinksidentification, viewcontentmcsidatamanagement, viewcontentvinsidatamanagement, viewcontentsidatamanagement, viewcontentmmedatamanagement</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>SourceKapture_Batches/&lt;module&gt;/dist/conf/application.properties -&gt; &lt;job folder&gt;/conf/application.properties</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Content store, folders, mail, run mode, logs</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>kapture.content.xml.root, *.reports.dir, vc.mail.to / *.notification.*, notification.smtp.*, batch.run.mode / batch.job.cron, logging.*</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>Content root /s3kapture/ROOT/resources/sites/KAPTURE/content; reports under .../library/MAZDA/GMS3_CUSTOM/... TBC: innerlinks.mdm.url (MDM web address on MC Dev), schedules (placeholders). The View Content jobs also create km_custom_batch_vc_sync in kapture_dc.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="100" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract job (newmgssexportjob.jar)</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>SourceCode_Migrated/NewMazdaDataExportTool/env/&lt;DEV|QA|PROD&gt;/application.properties (LOCAL = application.properties of the job folder) -&gt; dist/&lt;ENV&gt;/</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>DB, Kapture content, folders, transfer launch, mail</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>jdbc.conv.*, cms.table.article / .category, cms.state.*, kapture.article.date.format, kapture.content.xml.root, kapture.library.root, kapture.library.path.context, okassets.source.location.path, innerlink.kapture.pattern, othermanualink.kapture.url.pattern, wd.reflinks.kapture.pattern, mazda.content.extract.*, delete.csv.*, wd.js.files.temp.directory, transfer.job.*, NOTIF_EMAIL_*, SMTP_HOST_NAME</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>Added 2026-10-19. Every key required (exit 4 when missing). Log file: env/&lt;ENV&gt;/log.properties. Cron: hourly NORMAL + RERUN.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="50" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Transfer job (transferjob.jar)</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>SourceCode_Migrated/MazdaDataTransferTool/env/&lt;DEV|QA|PROD&gt;/application.properties (LOCAL = application.properties of the job folder) -&gt; dist/&lt;ENV&gt;/</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>DB, OCI Object Storage, folders, mail</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>jdbc.conv.*, oci.command, BUCKET_NAME, NAMESPACE, PROXY_URL, parallel.operations.count, mazda.content.extract.*, tansfer.reports.dir.path(.internal), delete.csv.*, NOTIF_EMAIL_*, SMTP_HOST_NAME</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>Added 2026-10-19. Started by the extract job (java -jar transferjob.jar &lt;jobId&gt; &lt;attemptId&gt; &lt;threadId&gt;); not scheduled itself.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="37.5" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>MGSS Bulk Data Extract - Run On Demand (newmgssrunondemandjob.jar)</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>SourceCode_Migrated/NewMazdaDataRunOnDemandTool/env/&lt;DEV|QA|PROD&gt;/application.properties (LOCAL = application.properties of the job folder) -&gt; dist/&lt;ENV&gt;/</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>DB, extract launch</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>jdbc.conv.*, extract.job.java.path, extract.job.location, xmxparam</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>Added 2026-10-19. Cron every few minutes; reads gms3_mdm_nmd_job_rod. NewMazdaDataReRunTool is replaced by a cron line (extract jar RERUN).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E25"/>
+  <autoFilter ref="A1:E27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4301,7 +4356,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -4311,7 +4366,7 @@
     <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Environment</t>
@@ -4503,7 +4558,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="25" customHeight="1">
+    <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>MC Dev</t>
@@ -4535,7 +4590,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="25" customHeight="1">
+    <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>MC Dev</t>
@@ -4567,7 +4622,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="25" customHeight="1">
+    <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>MC QA</t>
@@ -4612,7 +4667,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -4654,7 +4709,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1">
+    <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
           <t>kapture_cms_db.k_categories</t>
@@ -4686,7 +4741,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="25" customHeight="1">
+    <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>kapture_cms_db.k_article_comments</t>
@@ -4718,7 +4773,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="62.5" customHeight="1">
+    <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>kapture_cms_db.k_categories</t>
@@ -4859,7 +4914,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="25" customHeight="1">
+    <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>kapture_cms_db.k_article_recommendations</t>
@@ -4910,7 +4965,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="25" customHeight="1">
+    <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>kapture_cms_db.k_default_locales</t>

</xml_diff>